<commit_message>
Edited README.md to include instructions for setting up the virtual environment and installing dependencies. Updated drafting_script.py to modify the email body formatting and added comments for clarity. Updated login_script.py to clarify browser compatibility. Added .gitignore to exclude virtual environment and session files. Updated config.example.yaml to correct the path format for the Excel spreadsheet.
</commit_message>
<xml_diff>
--- a/Excel Spreadsheet Example/TasksSpreadsheetExample.xlsx
+++ b/Excel Spreadsheet Example/TasksSpreadsheetExample.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aliuddin\Documents\repos\Outlook-Drafting-Automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aliuddin\Documents\repos\Outlook-Drafting-Automation\Excel Spreadsheet Example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFF8D44C-480E-4A09-B65A-D2377040DC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB6F760-C90D-4855-9E4F-B97CFE890AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29940" yWindow="1140" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily_Tasks" sheetId="1" r:id="rId1"/>
@@ -399,6 +399,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -408,9 +411,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -498,6 +498,60 @@
           <bgColor rgb="FFC6E0B4"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -512,38 +566,6 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
@@ -594,28 +616,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -822,10 +822,10 @@
     <tableColumn id="3" xr3:uid="{89D09FB3-848F-4A6F-9330-24F45DEA5AF5}" name="Status" dataDxfId="16"/>
     <tableColumn id="4" xr3:uid="{74DFE9FF-97A5-4565-898F-F6A8E73F5337}" name="Report To" dataDxfId="15"/>
     <tableColumn id="5" xr3:uid="{B26E4F01-CFA8-48B4-9BBD-BF932CC44B20}" name="Start Date" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{0B046607-FEC5-41FB-B43D-3CA0F54DB877}" name="Due Date" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{6CFDAD3A-1877-4787-B005-3D7DA05A389B}" name="Remarks" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{0B046607-FEC5-41FB-B43D-3CA0F54DB877}" name="Due Date" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{6CFDAD3A-1877-4787-B005-3D7DA05A389B}" name="Remarks" dataDxfId="12"/>
     <tableColumn id="9" xr3:uid="{1F7E956C-8CF6-4390-AE11-CBEC8761719E}" name="Priority" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{402BE2EB-6B4C-43C0-9AF9-77CA9872F5D8}" name="Add To Email" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{402BE2EB-6B4C-43C0-9AF9-77CA9872F5D8}" name="Add To Email" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1156,16 +1156,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="16"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="17"/>
     </row>
     <row r="3" spans="1:12" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
@@ -1262,7 +1262,7 @@
       <c r="D6" s="3">
         <v>46281</v>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="14">
         <v>46283</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -1288,7 +1288,7 @@
       <c r="D7" s="3">
         <v>46282</v>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="14">
         <v>46308</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -1314,7 +1314,7 @@
       <c r="D8" s="3">
         <v>46283</v>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="14">
         <v>46290</v>
       </c>
       <c r="F8" s="2" t="s">

</xml_diff>

<commit_message>
Added new script for personal outlook accounts, renamed the script folders, added new information to the readme, and updated gitignore
</commit_message>
<xml_diff>
--- a/Excel Spreadsheet Example/TasksSpreadsheetExample.xlsx
+++ b/Excel Spreadsheet Example/TasksSpreadsheetExample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aliuddin\Documents\repos\Outlook-Drafting-Automation\Excel Spreadsheet Example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB6F760-C90D-4855-9E4F-B97CFE890AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3CD308-1082-4D82-9678-7109020075C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29940" yWindow="1140" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily_Tasks" sheetId="1" r:id="rId1"/>
@@ -105,9 +105,6 @@
     <t>to_recipient@example.com</t>
   </si>
   <si>
-    <t>cc_recipient@exampe.com</t>
-  </si>
-  <si>
     <t>Tasks</t>
   </si>
   <si>
@@ -154,6 +151,9 @@
   </si>
   <si>
     <t>Add</t>
+  </si>
+  <si>
+    <t>cc_recipient@example.com</t>
   </si>
 </sst>
 </file>
@@ -1157,7 +1157,7 @@
   <sheetData>
     <row r="2" spans="1:12" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -1175,7 +1175,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>2</v>
@@ -1190,7 +1190,7 @@
         <v>5</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
@@ -1201,7 +1201,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D4" s="3">
         <v>46279</v>
@@ -1210,10 +1210,10 @@
         <v>46279</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>14</v>
@@ -1231,7 +1231,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" s="3">
         <v>46280</v>
@@ -1240,10 +1240,10 @@
         <v>46280</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>14</v>
@@ -1254,10 +1254,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D6" s="3">
         <v>46281</v>
@@ -1266,13 +1266,13 @@
         <v>46283</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="46.5" x14ac:dyDescent="0.35">
@@ -1283,7 +1283,7 @@
         <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D7" s="3">
         <v>46282</v>
@@ -1292,13 +1292,13 @@
         <v>46308</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="31" x14ac:dyDescent="0.35">
@@ -1309,7 +1309,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D8" s="3">
         <v>46283</v>
@@ -1318,13 +1318,13 @@
         <v>46290</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1389,7 +1389,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2C9659-2315-4938-9E37-01407364AD81}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A2:A4"/>
+  <dimension ref="A2:A5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
@@ -1399,13 +1399,18 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" cm="1">
-        <f t="array" ref="A3:A4">_xlfn._xlws.FILTER(Daily_Tasks[No], Daily_Tasks[Add To Email]="Add", "")</f>
+        <f t="array" ref="A3:A5">_xlfn._xlws.FILTER(Daily_Tasks[No], Daily_Tasks[Add To Email]="Add", "")</f>
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1444,7 +1449,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Added extra code for popup removal in the personal script and added content into the readme.
</commit_message>
<xml_diff>
--- a/Excel Spreadsheet Example/TasksSpreadsheetExample.xlsx
+++ b/Excel Spreadsheet Example/TasksSpreadsheetExample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aliuddin\Documents\repos\Outlook-Drafting-Automation\Excel Spreadsheet Example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3CD308-1082-4D82-9678-7109020075C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B5CD2F7-D370-49AB-8055-1BB5642F23C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily_Tasks" sheetId="1" r:id="rId1"/>

</xml_diff>